<commit_message>
Corrida | SFE-MAQ | 2026-06-17 12:05:21.7536
</commit_message>
<xml_diff>
--- a/indicadores/SFE-MAQ_out.xlsx
+++ b/indicadores/SFE-MAQ_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="526">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Producción de maquinaria agrícola en Santa Fe</t>
+    <t xml:space="preserve">Producción de maquinaria agrícola</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -74,6 +74,12 @@
     <t xml:space="preserve">const</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -107,13 +113,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2088,9 +2094,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>19</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2101,7 +2111,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2115,7 +2125,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2131,7 +2141,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2159,7 +2169,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2173,7 +2183,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2201,7 +2211,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2215,7 +2225,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2229,7 +2239,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2243,7 +2253,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2259,7 +2269,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2273,7 +2283,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2421,10 +2431,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2437,10 +2447,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2464,66 +2474,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="J1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="M1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="N1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="P1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="Q1" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="R1" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="S1" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>49.2291346931581</v>
@@ -2576,7 +2586,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>70.1963223469226</v>
@@ -2633,7 +2643,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>95.9172551565845</v>
@@ -2690,7 +2700,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>93.331067988469</v>
@@ -2747,7 +2757,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>71.7246433296081</v>
@@ -2804,7 +2814,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>51.1016727700635</v>
@@ -2861,7 +2871,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>46.6336664129265</v>
@@ -2918,7 +2928,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>43.7750458031266</v>
@@ -2975,7 +2985,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>37.639175403193</v>
@@ -3032,7 +3042,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>72.6855109597325</v>
@@ -3089,7 +3099,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>63.2431516219355</v>
@@ -3146,7 +3156,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>71.6502312434944</v>
@@ -3203,7 +3213,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>55.3583524145537</v>
@@ -3262,7 +3272,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>75.4072169429994</v>
@@ -3321,7 +3331,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>98.2761818213992</v>
@@ -3380,7 +3390,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>139.811885984208</v>
@@ -3439,7 +3449,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>110.032294885627</v>
@@ -3498,7 +3508,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>76.2710860178184</v>
@@ -3557,7 +3567,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>62.0364612642782</v>
@@ -3616,7 +3626,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>127.300975135346</v>
@@ -3675,7 +3685,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>129.815378650926</v>
@@ -3734,7 +3744,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>129.522987173628</v>
@@ -3793,7 +3803,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>106.76432620761</v>
@@ -3852,7 +3862,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>103.185403828062</v>
@@ -3911,7 +3921,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>62.9348263539833</v>
@@ -3970,7 +3980,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>77.6917315217006</v>
@@ -4029,7 +4039,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>149.682155614455</v>
@@ -4088,7 +4098,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>156.509088636407</v>
@@ -4147,7 +4157,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>92.4393555773018</v>
@@ -4206,7 +4216,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>65.8718832948566</v>
@@ -4265,7 +4275,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>78.3934710672164</v>
@@ -4324,7 +4334,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>84.4216659883467</v>
@@ -4383,7 +4393,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>89.5129755599261</v>
@@ -4442,7 +4452,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>123.893463397218</v>
@@ -4501,7 +4511,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>79.0871621228127</v>
@@ -4560,7 +4570,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>83.0847136826943</v>
@@ -4619,7 +4629,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>65.0731451940352</v>
@@ -4678,7 +4688,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>80.9623286332963</v>
@@ -4737,7 +4747,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>162.345914880504</v>
@@ -4796,7 +4806,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>154.033205380673</v>
@@ -4855,7 +4865,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>79.9762461004017</v>
@@ -4914,7 +4924,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>39.3881042106412</v>
@@ -4973,7 +4983,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>37.2271989013973</v>
@@ -5032,7 +5042,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>57.8183018796338</v>
@@ -5091,7 +5101,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>52.1462335984177</v>
@@ -5150,7 +5160,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>85.7971385538451</v>
@@ -5209,7 +5219,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>57.9671260518611</v>
@@ -5268,7 +5278,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>56.7178911893981</v>
@@ -5327,7 +5337,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>48.1938549769199</v>
@@ -5386,7 +5396,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>55.7043034192002</v>
@@ -5445,7 +5455,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>68.4147525028391</v>
@@ -5504,7 +5514,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>74.4168631024756</v>
@@ -5563,7 +5573,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>59.2636517917804</v>
@@ -5622,7 +5632,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>41.9196728993986</v>
@@ -5681,7 +5691,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>38.1172427755405</v>
@@ -5740,7 +5750,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>36.9664753221256</v>
@@ -5799,7 +5809,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>44.1067191682775</v>
@@ -5858,7 +5868,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>59.7647005455669</v>
@@ -5917,7 +5927,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>43.5566038553692</v>
@@ -5976,7 +5986,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>34.4798381172316</v>
@@ -6035,7 +6045,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>17.3261531041981</v>
@@ -6094,7 +6104,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>25.4573305194999</v>
@@ -6153,7 +6163,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>54.6152367318066</v>
@@ -6212,7 +6222,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>68.2876296579885</v>
@@ -6271,7 +6281,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>63.4489207186664</v>
@@ -6330,7 +6340,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>33.8301194176032</v>
@@ -6389,7 +6399,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>36.4364368417322</v>
@@ -6448,7 +6458,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>36.345746349104</v>
@@ -6507,7 +6517,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>32.3091473680599</v>
@@ -6566,7 +6576,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>52.5263235811713</v>
@@ -6625,7 +6635,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>53.3447890591567</v>
@@ -6684,7 +6694,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>57.1672960155297</v>
@@ -6743,7 +6753,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>17.5112554022623</v>
@@ -6802,7 +6812,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>34.9660016197873</v>
@@ -6861,7 +6871,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>48.0176655729476</v>
@@ -6920,7 +6930,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>68.991606498023</v>
@@ -6979,7 +6989,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>52.4118349432205</v>
@@ -7038,7 +7048,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>32.7536869371092</v>
@@ -7097,7 +7107,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>31.4378940181451</v>
@@ -7156,7 +7166,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>24.0634813148072</v>
@@ -7215,7 +7225,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>29.6299652394864</v>
@@ -7274,7 +7284,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>56.9710297790425</v>
@@ -7333,7 +7343,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>46.0900565750538</v>
@@ -7392,7 +7402,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>25.9799263742779</v>
@@ -7451,7 +7461,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>20.7799257329193</v>
@@ -7510,7 +7520,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>19.8188554791693</v>
@@ -7569,7 +7579,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>18.2386172303812</v>
@@ -7628,7 +7638,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>44.2674826190306</v>
@@ -7687,7 +7697,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>40.9145279487497</v>
@@ -7746,7 +7756,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>38.5888525166853</v>
@@ -7805,7 +7815,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>60.8348549549832</v>
@@ -7864,7 +7874,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>59.0448823758368</v>
@@ -7923,7 +7933,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>58.1430146109865</v>
@@ -7982,7 +7992,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>83.790284619863</v>
@@ -8041,7 +8051,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>83.7417764193608</v>
@@ -8100,7 +8110,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>83.3846332737289</v>
@@ -8159,7 +8169,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>81.2052659433587</v>
@@ -8218,7 +8228,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>80.3037474566719</v>
@@ -8277,7 +8287,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>79.822040685937</v>
@@ -8336,7 +8346,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>103.016365879837</v>
@@ -8395,7 +8405,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>103.321985922269</v>
@@ -8454,7 +8464,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>103.371358943323</v>
@@ -8513,7 +8523,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>137.046798708203</v>
@@ -8572,7 +8582,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>138.142100752852</v>
@@ -8631,7 +8641,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>138.156963999546</v>
@@ -8690,7 +8700,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>174.118897617357</v>
@@ -8749,7 +8759,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>173.289184079282</v>
@@ -8808,7 +8818,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>172.01373850155</v>
@@ -8867,7 +8877,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>172.81645420851</v>
@@ -8926,7 +8936,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>171.361435633899</v>
@@ -8985,7 +8995,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>170.22146291003</v>
@@ -9044,7 +9054,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>163.114954686342</v>
@@ -9103,7 +9113,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>162.262704456264</v>
@@ -9162,7 +9172,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>161.339342359657</v>
@@ -9221,7 +9231,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>164.738532759664</v>
@@ -9280,7 +9290,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>162.91759074104</v>
@@ -9339,7 +9349,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>161.882380030914</v>
@@ -9398,7 +9408,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>185.160582216186</v>
@@ -9457,7 +9467,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>186.054324802153</v>
@@ -9516,7 +9526,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>185.56138320084</v>
@@ -9575,7 +9585,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>139.208185219326</v>
@@ -9634,7 +9644,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>136.469420578636</v>
@@ -9693,7 +9703,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>133.439392810959</v>
@@ -9752,7 +9762,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>132.849565771376</v>
@@ -9811,7 +9821,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>132.616671721724</v>
@@ -9870,7 +9880,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>132.473183489986</v>
@@ -9929,7 +9939,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>155.6953475683</v>
@@ -9988,7 +9998,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>153.816435006122</v>
@@ -10047,7 +10057,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>153.104417661901</v>
@@ -10106,7 +10116,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>189.083686476335</v>
@@ -10165,7 +10175,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>186.906999379604</v>
@@ -10224,7 +10234,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>185.509475818755</v>
@@ -10283,7 +10293,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>128.109705717104</v>
@@ -10342,7 +10352,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>79.5371716815202</v>
@@ -10401,7 +10411,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>83.5780011261428</v>
@@ -10460,7 +10470,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>133.326828239086</v>
@@ -10519,7 +10529,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>84.9236973921165</v>
@@ -10578,7 +10588,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>72.0764290890137</v>
@@ -10637,7 +10647,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>81.3385231186835</v>
@@ -10696,7 +10706,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>129.237474591857</v>
@@ -10755,7 +10765,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>108.809304012901</v>
@@ -10814,7 +10824,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>110.92824176062</v>
@@ -10873,7 +10883,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>81.0684265154011</v>
@@ -10932,7 +10942,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>107.066196755555</v>
@@ -10991,7 +11001,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>90.9259027411415</v>
@@ -11050,7 +11060,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>89.673007875975</v>
@@ -11109,7 +11119,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>83.0177619548978</v>
@@ -11168,7 +11178,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>74.118841557694</v>
@@ -11227,7 +11237,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>121.836744828145</v>
@@ -11286,7 +11296,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>109.044102632466</v>
@@ -11345,7 +11355,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>125.288326281044</v>
@@ -11404,7 +11414,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>123.599588978497</v>
@@ -11463,7 +11473,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>112.853302006028</v>
@@ -11522,7 +11532,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>104.31624974183</v>
@@ -11581,7 +11591,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>157.298858608463</v>
@@ -11640,7 +11650,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>122.21869575305</v>
@@ -11699,7 +11709,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>93.8477388099053</v>
@@ -11758,7 +11768,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>117.857803386456</v>
@@ -11817,7 +11827,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>94.503134625988</v>
@@ -11876,7 +11886,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>185.950752973731</v>
@@ -11935,7 +11945,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>167.127140489776</v>
@@ -11994,7 +12004,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>79.0543898477379</v>
@@ -12053,7 +12063,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>157.899099449699</v>
@@ -12112,7 +12122,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>119.806981333377</v>
@@ -12171,7 +12181,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>156.093877785119</v>
@@ -12230,7 +12240,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>101.268273860778</v>
@@ -12289,7 +12299,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>129.739565253541</v>
@@ -12348,7 +12358,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>134.03310810832</v>
@@ -12407,7 +12417,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>78.9167560921636</v>
@@ -12466,7 +12476,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>70.7513447099727</v>
@@ -12525,7 +12535,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>48.794463156756</v>
@@ -12584,7 +12594,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>69.4895668136304</v>
@@ -12643,7 +12653,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>71.4315903605591</v>
@@ -12702,7 +12712,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>121.733751298443</v>
@@ -12761,7 +12771,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>63.6815549072865</v>
@@ -12820,7 +12830,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>82.4778895179315</v>
@@ -12879,7 +12889,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>70.9312499012292</v>
@@ -12938,7 +12948,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>68.1662072657281</v>
@@ -12997,7 +13007,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>74.7420249951793</v>
@@ -13056,7 +13066,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>92.6797961290946</v>
@@ -13115,7 +13125,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>135.643002690616</v>
@@ -13174,7 +13184,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>59.7849054759239</v>
@@ -13233,7 +13243,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>57.5055329560738</v>
@@ -13292,7 +13302,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>113.090631586268</v>
@@ -13351,7 +13361,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>96.6348441221441</v>
@@ -13410,7 +13420,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>109.986151710622</v>
@@ -13469,7 +13479,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>97.2164084668158</v>
@@ -13528,7 +13538,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>91.7961192743089</v>
@@ -13587,7 +13597,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>130.885552083572</v>
@@ -13646,7 +13656,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>83.3075074399188</v>
@@ -13705,7 +13715,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>131.42036036476</v>
@@ -13764,7 +13774,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>147.722555122565</v>
@@ -13823,7 +13833,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>89.6072324790753</v>
@@ -13882,7 +13892,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>112.891083691209</v>
@@ -13941,7 +13951,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>103.201938393929</v>
@@ -14000,7 +14010,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>135.40815698085</v>
@@ -14059,7 +14069,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>114.739956765332</v>
@@ -14118,7 +14128,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>122.120490279343</v>
@@ -14177,7 +14187,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>243.354419094638</v>
@@ -14236,7 +14246,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>101.824290530159</v>
@@ -14295,7 +14305,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>107.319711652064</v>
@@ -14354,7 +14364,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>78.2788972384529</v>
@@ -14413,7 +14423,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>109.532696122766</v>
@@ -14472,7 +14482,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>116.796530500282</v>
@@ -14531,7 +14541,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>48.7809467551875</v>
@@ -14590,7 +14600,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>175.200434129907</v>
@@ -14649,7 +14659,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>99.7622593549426</v>
@@ -14708,7 +14718,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>92.5723133832446</v>
@@ -14767,7 +14777,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>98.1796400469593</v>
@@ -14826,7 +14836,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>112.622377066481</v>
@@ -14885,7 +14895,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>84.0216414473882</v>
@@ -14944,7 +14954,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>120.310176019941</v>
@@ -15003,7 +15013,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>92.5143816389248</v>
@@ -15062,7 +15072,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>120.776582315841</v>
@@ -15121,7 +15131,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>92.4024374574544</v>
@@ -15180,7 +15190,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>136.327576241699</v>
@@ -15239,7 +15249,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>53.9690018152535</v>
@@ -15298,7 +15308,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>68.0877897412241</v>
@@ -15357,7 +15367,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>122.259722291554</v>
@@ -15416,7 +15426,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>77.3170565205515</v>
@@ -15475,7 +15485,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>108.00819645017</v>
@@ -15534,7 +15544,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>172.152354002716</v>
@@ -15593,7 +15603,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>132.383575697435</v>
@@ -15652,7 +15662,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>97.6801141946778</v>
@@ -15711,7 +15721,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>121.903179530147</v>
@@ -15770,7 +15780,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>107.481165881595</v>
@@ -15829,7 +15839,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>137.756305360555</v>
@@ -15888,7 +15898,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>230.879088934185</v>
@@ -15947,7 +15957,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>61.9722903723983</v>
@@ -16006,7 +16016,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>79.5387475271873</v>
@@ -16065,7 +16075,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>82.1081297296591</v>
@@ -16124,7 +16134,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>101.330902615254</v>
@@ -16183,7 +16193,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>88.2121794262126</v>
@@ -16242,7 +16252,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>143.1207136198</v>
@@ -16301,7 +16311,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>93.3293831361122</v>
@@ -16360,7 +16370,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>77.159487130553</v>
@@ -16419,7 +16429,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>104.466612242327</v>
@@ -16478,7 +16488,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>107.41391941259</v>
@@ -16537,7 +16547,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>103.152491342544</v>
@@ -16596,7 +16606,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>114.601560255794</v>
@@ -16655,7 +16665,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>64.30244693117</v>
@@ -16714,7 +16724,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>73.9050418696305</v>
@@ -16773,7 +16783,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>101.251173571398</v>
@@ -16832,7 +16842,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>113.0795499743</v>
@@ -16891,7 +16901,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>89.5177491137575</v>
@@ -16950,7 +16960,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>158.51591921849</v>
@@ -17009,7 +17019,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>74.3954815349432</v>
@@ -17068,7 +17078,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>78.2390759060628</v>
@@ -17127,7 +17137,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>114.619205598999</v>
@@ -17186,7 +17196,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>106.497717741929</v>
@@ -17245,7 +17255,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>141.568485656117</v>
@@ -17304,7 +17314,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>158.798069427342</v>
@@ -17363,7 +17373,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>53.3458757102158</v>
@@ -17422,7 +17432,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>65.0258314510931</v>
@@ -17481,7 +17491,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>105.934204150721</v>
@@ -17540,7 +17550,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>94.2967270421549</v>
@@ -17599,7 +17609,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>99.7149589405116</v>
@@ -17658,7 +17668,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>82.9967714472906</v>
@@ -17717,7 +17727,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>97.2648906015305</v>
@@ -17776,7 +17786,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>174.001996669291</v>
@@ -17835,7 +17845,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>187.443749589934</v>
@@ -17894,7 +17904,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>140.392459213918</v>
@@ -17953,7 +17963,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>199.801813388429</v>
@@ -18012,7 +18022,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>176.220628098138</v>
@@ -18071,7 +18081,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>94.098677395437</v>
@@ -18130,7 +18140,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>139.965413333169</v>
@@ -18189,7 +18199,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>166.022056053356</v>
@@ -18248,7 +18258,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>154.426598412986</v>
@@ -18307,7 +18317,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>165.614681498741</v>
@@ -18366,7 +18376,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>147.348717572996</v>
@@ -18425,7 +18435,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>111.179287547348</v>
@@ -18484,7 +18494,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>130.944704768253</v>
@@ -18543,7 +18553,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>141.454348572479</v>
@@ -18602,7 +18612,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>172.229503490719</v>
@@ -18661,7 +18671,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>144.09108900889</v>
@@ -18720,7 +18730,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>216.330484606985</v>
@@ -18779,7 +18789,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>137.227496352194</v>
@@ -18838,7 +18848,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>148.850318219493</v>
@@ -18897,7 +18907,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>152.445002800727</v>
@@ -18956,7 +18966,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>152.16527628068</v>
@@ -19015,7 +19025,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>144.216601497774</v>
@@ -19074,7 +19084,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>123.566399795863</v>
@@ -19133,7 +19143,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>123.550195504162</v>
@@ -19192,7 +19202,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>128.613407311323</v>
@@ -19251,7 +19261,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>99.8283791917696</v>
@@ -19310,7 +19320,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>125.879870228243</v>
@@ -19369,7 +19379,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>105.472226625836</v>
@@ -19428,7 +19438,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>109.122691796841</v>
@@ -19487,7 +19497,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>106.6130192639</v>
@@ -19546,7 +19556,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>124.822712755153</v>
@@ -19605,7 +19615,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>123.453171590311</v>
@@ -19664,7 +19674,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>109.203125406414</v>
@@ -19723,7 +19733,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>102.116996127243</v>
@@ -19782,7 +19792,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>100.870869295131</v>
@@ -19841,7 +19851,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>110.979389209699</v>
@@ -19900,7 +19910,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>123.682869829877</v>
@@ -19959,7 +19969,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>121.436584426143</v>
@@ -20018,7 +20028,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>148.614993056002</v>
@@ -20077,7 +20087,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>107.367403307135</v>
@@ -20136,7 +20146,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>97.3080579612002</v>
@@ -20195,7 +20205,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>97.8685535831965</v>
@@ -20254,7 +20264,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>93.5117064373034</v>
@@ -20313,7 +20323,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>101.759939844712</v>
@@ -20372,7 +20382,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>114.272395708364</v>
@@ -20431,7 +20441,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>121.944194942291</v>
@@ -20490,7 +20500,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>142.215434352638</v>
@@ -20549,7 +20559,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>121.923922532768</v>
@@ -20608,7 +20618,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>151.214534594615</v>
@@ -20667,7 +20677,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>152.474214592979</v>
@@ -20726,7 +20736,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>159.119593519063</v>
@@ -20785,7 +20795,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>149.901767095726</v>
@@ -20844,7 +20854,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>152.931561084578</v>
@@ -20903,7 +20913,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>97.070332185421</v>
@@ -20962,7 +20972,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>109.890942096703</v>
@@ -21021,7 +21031,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>167.583686697472</v>
@@ -21080,7 +21090,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>108.975184245897</v>
@@ -21139,7 +21149,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>105.312152842674</v>
@@ -21198,7 +21208,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>141.026709024102</v>
@@ -21257,7 +21267,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>171.246718100696</v>
@@ -21316,7 +21326,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>171.246718100696</v>
@@ -21375,7 +21385,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>171.246718100696</v>
@@ -21434,7 +21444,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>208.792789983736</v>
@@ -21493,7 +21503,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>210.624305685347</v>
@@ -21552,7 +21562,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>163.920655294249</v>
@@ -21611,7 +21621,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>133.700646217655</v>
@@ -21670,7 +21680,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>117.21700490315</v>
@@ -21729,7 +21739,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>111.722457798315</v>
@@ -21788,7 +21798,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>175.825507354725</v>
@@ -21847,7 +21857,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>205.129758580512</v>
@@ -21906,7 +21916,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>168.499444548278</v>
@@ -21965,7 +21975,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>205.129758580512</v>
@@ -22024,7 +22034,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>209.708547834542</v>
@@ -22083,7 +22093,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>177.657023056337</v>
@@ -22142,7 +22152,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>144.689740427326</v>
@@ -22201,7 +22211,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>140.110951173296</v>
@@ -22260,7 +22270,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>133.700646217655</v>
@@ -22319,7 +22329,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>125.458825560403</v>
@@ -22378,7 +22388,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>102.564879290256</v>
@@ -22437,7 +22447,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>143.77398257652</v>
@@ -22496,7 +22506,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>142.858224725714</v>
@@ -22555,7 +22565,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>146.521256128937</v>
@@ -22614,7 +22624,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>109.890942096703</v>
@@ -22673,7 +22683,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>140.110951173296</v>
@@ -22732,7 +22742,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>140.110951173296</v>
@@ -22791,7 +22801,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>125.458825560403</v>
@@ -22850,7 +22860,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>126.374583411209</v>
@@ -22909,7 +22919,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>124.543067709597</v>
@@ -22968,7 +22978,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>107.143668544285</v>
@@ -23027,7 +23037,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>80.5866908709156</v>
@@ -23086,7 +23096,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>67.7660809596336</v>
@@ -23145,7 +23155,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>65.018807407216</v>
@@ -23204,7 +23214,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>97.070332185421</v>
@@ -23263,7 +23273,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>125.458825560403</v>
@@ -23322,7 +23332,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>74.1763859152746</v>
@@ -23381,7 +23391,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>146.521256128937</v>
@@ -23440,7 +23450,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>228.939462701465</v>
@@ -23499,7 +23509,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>158.426108189414</v>
@@ -23558,7 +23568,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>172.162475951501</v>
@@ -23617,7 +23627,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>163.004897443443</v>
@@ -23676,7 +23686,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>155.678834636996</v>
@@ -23735,7 +23745,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>173.993991653113</v>
@@ -23794,7 +23804,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>146.521256128937</v>
@@ -23853,7 +23863,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>132.78488836685</v>
@@ -23912,7 +23922,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>216.118852790183</v>
@@ -23971,7 +23981,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>252.749166822417</v>
@@ -24030,7 +24040,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>184.067328011978</v>
@@ -24089,7 +24099,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>208.792789983736</v>
@@ -24148,7 +24158,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>205.129758580512</v>
@@ -24207,7 +24217,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>226.192189149047</v>
@@ -24266,7 +24276,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>206.045516431318</v>
@@ -24325,7 +24335,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>173.993991653113</v>
@@ -24384,7 +24394,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>137.363677620879</v>
@@ -24443,7 +24453,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>154.76307678619</v>
@@ -24502,7 +24512,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>132.784888366849</v>
@@ -24561,7 +24571,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>150.184287532161</v>
@@ -24620,7 +24630,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>239.012799060329</v>
@@ -24679,7 +24689,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>246.338861866776</v>
@@ -24738,7 +24748,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B379" s="2"/>
       <c r="C379" s="3" t="n">
@@ -24771,7 +24781,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B380" s="2"/>
       <c r="C380" s="3" t="n">
@@ -24804,7 +24814,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B381" s="2"/>
       <c r="C381" s="3" t="n">
@@ -24837,7 +24847,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B382" s="2"/>
       <c r="C382" s="3" t="n">
@@ -24870,7 +24880,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B383" s="2"/>
       <c r="C383" s="3" t="n">
@@ -24903,7 +24913,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B384" s="2"/>
       <c r="C384" s="3" t="n">
@@ -24936,7 +24946,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B385" s="2"/>
       <c r="C385" s="3" t="n">
@@ -24969,7 +24979,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B386" s="2"/>
       <c r="C386" s="3" t="n">
@@ -25002,7 +25012,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B387" s="2"/>
       <c r="C387" s="3" t="n">
@@ -25035,7 +25045,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B388" s="2"/>
       <c r="C388" s="3" t="n">
@@ -25068,7 +25078,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B389" s="2"/>
       <c r="C389" s="3" t="n">
@@ -25101,7 +25111,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3" t="n">
@@ -25134,7 +25144,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3"/>
@@ -25157,7 +25167,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3"/>
@@ -25180,7 +25190,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3"/>
@@ -25203,7 +25213,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3"/>
@@ -25226,7 +25236,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3"/>
@@ -25249,7 +25259,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3"/>
@@ -25272,7 +25282,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3"/>
@@ -25295,7 +25305,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3"/>
@@ -25318,7 +25328,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3"/>
@@ -25341,7 +25351,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3"/>
@@ -25364,7 +25374,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3"/>
@@ -25387,7 +25397,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -25410,7 +25420,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25433,7 +25443,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25456,7 +25466,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25479,7 +25489,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25502,7 +25512,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25525,7 +25535,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25548,7 +25558,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25571,7 +25581,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25594,7 +25604,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -25617,7 +25627,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -25640,7 +25650,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -25663,7 +25673,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -25686,7 +25696,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -25709,7 +25719,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -25732,7 +25742,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -25755,7 +25765,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -25778,7 +25788,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -25801,7 +25811,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -25824,7 +25834,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -25847,7 +25857,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -25870,7 +25880,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -25893,7 +25903,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -25916,7 +25926,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -25939,7 +25949,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -25962,7 +25972,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -25985,7 +25995,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26008,7 +26018,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26031,7 +26041,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26054,7 +26064,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26077,7 +26087,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26100,7 +26110,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26134,97 +26144,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
   </sheetData>
@@ -26248,7 +26258,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -26258,13 +26268,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>0.0707864050319593</v>
@@ -26272,7 +26282,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>0.0874346774436116</v>
@@ -26280,7 +26290,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>0.135105075373629</v>
@@ -26288,7 +26298,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.186096485284369</v>
@@ -26296,7 +26306,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>0.224877793112315</v>
@@ -26304,7 +26314,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>0.255627525533043</v>
@@ -26312,7 +26322,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>0.221756435239215</v>
@@ -26320,7 +26330,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>0.183448996759789</v>
@@ -26328,7 +26338,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.187016756551444</v>
@@ -26336,7 +26346,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.176559163022594</v>
@@ -26344,7 +26354,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.144604929325258</v>
@@ -26352,7 +26362,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>0.103311683129267</v>
@@ -26360,7 +26370,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>0.0508067386308981</v>
@@ -26368,7 +26378,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>-0.0106542774565447</v>
@@ -26376,7 +26386,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.0890271359844208</v>
@@ -26384,7 +26394,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>-0.169464317111368</v>
@@ -26392,7 +26402,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>-0.204477263225228</v>
@@ -26400,7 +26410,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>-0.212971199929736</v>
@@ -26408,7 +26418,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>-0.238989393070842</v>

</xml_diff>